<commit_message>
BA rows mapped to SOES213 (BSc-only) moved to SOES226
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/20261013_CurriculumMapping_Geography.xlsx
+++ b/curriculum_mapping_2026-27/20261013_CurriculumMapping_Geography.xlsx
@@ -16893,7 +16893,7 @@
       </c>
       <c r="C273" s="9" t="inlineStr">
         <is>
-          <t>SOES213 GEOGRAPHICAL DATA ANALYSIS AND PROCESSING</t>
+          <t>SOES226 EXPLORING THE SOCIAL WORLD</t>
         </is>
       </c>
       <c r="D273" s="9" t="inlineStr">
@@ -26013,7 +26013,7 @@
       </c>
       <c r="C463" s="9" t="inlineStr">
         <is>
-          <t>SOES213 GEOGRAPHICAL DATA ANALYSIS AND PROCESSING</t>
+          <t>SOES226 EXPLORING THE SOCIAL WORLD</t>
         </is>
       </c>
       <c r="D463" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Core/optional column: Core for rows matched to UoL compulsory modules
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/20261013_CurriculumMapping_Geography.xlsx
+++ b/curriculum_mapping_2026-27/20261013_CurriculumMapping_Geography.xlsx
@@ -4433,7 +4433,7 @@
       </c>
       <c r="G13" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H13" s="9" t="inlineStr">
@@ -5537,7 +5537,7 @@
       </c>
       <c r="G36" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H36" s="9" t="inlineStr">
@@ -6209,7 +6209,7 @@
       </c>
       <c r="G50" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H50" s="9" t="inlineStr">
@@ -6401,7 +6401,7 @@
       </c>
       <c r="G54" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H54" s="9" t="inlineStr">
@@ -10721,7 +10721,7 @@
       </c>
       <c r="G144" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H144" s="9" t="inlineStr">
@@ -10913,7 +10913,7 @@
       </c>
       <c r="G148" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H148" s="9" t="inlineStr">
@@ -12065,7 +12065,7 @@
       </c>
       <c r="G172" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H172" s="9" t="inlineStr">
@@ -14705,7 +14705,7 @@
       </c>
       <c r="G227" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H227" s="9" t="inlineStr">
@@ -14849,7 +14849,7 @@
       </c>
       <c r="G230" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H230" s="9" t="inlineStr">
@@ -15473,7 +15473,7 @@
       </c>
       <c r="G243" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H243" s="9" t="inlineStr">
@@ -16097,7 +16097,7 @@
       </c>
       <c r="G256" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H256" s="9" t="inlineStr">
@@ -16289,7 +16289,7 @@
       </c>
       <c r="G260" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H260" s="9" t="inlineStr">
@@ -16913,7 +16913,7 @@
       </c>
       <c r="G273" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H273" s="9" t="inlineStr">
@@ -16961,7 +16961,7 @@
       </c>
       <c r="G274" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H274" s="9" t="inlineStr">
@@ -18065,7 +18065,7 @@
       </c>
       <c r="G297" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H297" s="9" t="inlineStr">
@@ -18161,7 +18161,7 @@
       </c>
       <c r="G299" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H299" s="9" t="inlineStr">
@@ -18593,7 +18593,7 @@
       </c>
       <c r="G308" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H308" s="9" t="inlineStr">
@@ -20417,7 +20417,7 @@
       </c>
       <c r="G346" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H346" s="9" t="inlineStr">
@@ -23585,7 +23585,7 @@
       </c>
       <c r="G412" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H412" s="9" t="inlineStr">
@@ -23921,7 +23921,7 @@
       </c>
       <c r="G419" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H419" s="9" t="inlineStr">
@@ -24737,7 +24737,7 @@
       </c>
       <c r="G436" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H436" s="9" t="inlineStr">
@@ -25025,7 +25025,7 @@
       </c>
       <c r="G442" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H442" s="9" t="inlineStr">
@@ -25601,7 +25601,7 @@
       </c>
       <c r="G454" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H454" s="9" t="inlineStr">
@@ -26033,7 +26033,7 @@
       </c>
       <c r="G463" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H463" s="9" t="inlineStr">
@@ -26081,7 +26081,7 @@
       </c>
       <c r="G464" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H464" s="9" t="inlineStr">
@@ -28481,7 +28481,7 @@
       </c>
       <c r="G514" s="9" t="inlineStr">
         <is>
-          <t>Optional</t>
+          <t>Core</t>
         </is>
       </c>
       <c r="H514" s="9" t="inlineStr">

</xml_diff>

<commit_message>
Column K: SOES213 corresponds to ENVS202 Key Skills for Environmental Data Analysis
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/20261013_CurriculumMapping_Geography.xlsx
+++ b/curriculum_mapping_2026-27/20261013_CurriculumMapping_Geography.xlsx
@@ -4828,7 +4828,7 @@
       <c r="J19" s="9" t="n"/>
       <c r="K19" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -11665,7 +11665,7 @@
       <c r="J148" s="9" t="n"/>
       <c r="K148" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -16011,7 +16011,7 @@
       <c r="J230" s="9" t="n"/>
       <c r="K230" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -16700,7 +16700,7 @@
       <c r="J243" s="9" t="n"/>
       <c r="K243" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -17601,7 +17601,7 @@
       <c r="J260" s="9" t="n"/>
       <c r="K260" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -18343,7 +18343,7 @@
       <c r="J274" s="9" t="n"/>
       <c r="K274" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -19562,7 +19562,7 @@
       <c r="J297" s="9" t="n"/>
       <c r="K297" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -19668,7 +19668,7 @@
       <c r="J299" s="9" t="n"/>
       <c r="K299" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -22795,7 +22795,7 @@
       <c r="J358" s="9" t="n"/>
       <c r="K358" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -26876,7 +26876,7 @@
       <c r="J435" s="9" t="n"/>
       <c r="K435" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -27406,7 +27406,7 @@
       <c r="J445" s="9" t="n"/>
       <c r="K445" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>
@@ -28042,7 +28042,7 @@
       <c r="J457" s="9" t="n"/>
       <c r="K457" s="9" t="inlineStr">
         <is>
-          <t>No direct 2026/27 equivalent (new module)</t>
+          <t>ENVS202 Key Skills for Environmental Data Analysis (closest)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Column K: apply confirmed SOES-ENVS correspondences
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/20261013_CurriculumMapping_Geography.xlsx
+++ b/curriculum_mapping_2026-27/20261013_CurriculumMapping_Geography.xlsx
@@ -3976,7 +3976,7 @@
       <c r="J3" s="10" t="n"/>
       <c r="K3" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -4029,7 +4029,7 @@
       <c r="J4" s="10" t="n"/>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -4082,7 +4082,7 @@
       <c r="J5" s="10" t="n"/>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -4135,7 +4135,7 @@
       <c r="J6" s="10" t="n"/>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -4241,7 +4241,7 @@
       <c r="J8" s="9" t="n"/>
       <c r="K8" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -4347,7 +4347,7 @@
       <c r="J10" s="9" t="n"/>
       <c r="K10" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -4453,7 +4453,7 @@
       <c r="J12" s="9" t="n"/>
       <c r="K12" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -4506,7 +4506,7 @@
       <c r="J13" s="9" t="n"/>
       <c r="K13" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -4718,7 +4718,7 @@
       <c r="J17" s="9" t="n"/>
       <c r="K17" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -4771,7 +4771,7 @@
       <c r="J18" s="9" t="n"/>
       <c r="K18" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -4824,7 +4824,7 @@
       <c r="J19" s="9" t="n"/>
       <c r="K19" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -5089,7 +5089,7 @@
       <c r="J24" s="9" t="n"/>
       <c r="K24" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -5142,7 +5142,7 @@
       <c r="J25" s="9" t="n"/>
       <c r="K25" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -5460,7 +5460,7 @@
       <c r="J31" s="9" t="n"/>
       <c r="K31" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -5513,7 +5513,7 @@
       <c r="J32" s="9" t="n"/>
       <c r="K32" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -5566,7 +5566,7 @@
       <c r="J33" s="9" t="n"/>
       <c r="K33" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -5672,7 +5672,7 @@
       <c r="J35" s="9" t="n"/>
       <c r="K35" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -5725,7 +5725,7 @@
       <c r="J36" s="9" t="n"/>
       <c r="K36" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -5778,7 +5778,7 @@
       <c r="J37" s="9" t="n"/>
       <c r="K37" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -5937,7 +5937,7 @@
       <c r="J40" s="9" t="n"/>
       <c r="K40" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -6149,7 +6149,7 @@
       <c r="J44" s="9" t="n"/>
       <c r="K44" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -6414,7 +6414,7 @@
       <c r="J49" s="9" t="n"/>
       <c r="K49" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -6467,7 +6467,7 @@
       <c r="J50" s="9" t="n"/>
       <c r="K50" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -6520,7 +6520,7 @@
       <c r="J51" s="9" t="n"/>
       <c r="K51" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -6626,7 +6626,7 @@
       <c r="J53" s="9" t="n"/>
       <c r="K53" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -6679,7 +6679,7 @@
       <c r="J54" s="9" t="n"/>
       <c r="K54" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -6732,7 +6732,7 @@
       <c r="J55" s="9" t="n"/>
       <c r="K55" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -6785,7 +6785,7 @@
       <c r="J56" s="9" t="n"/>
       <c r="K56" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -6838,7 +6838,7 @@
       <c r="J57" s="9" t="n"/>
       <c r="K57" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -6997,7 +6997,7 @@
       <c r="J60" s="9" t="n"/>
       <c r="K60" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -7103,7 +7103,7 @@
       <c r="J62" s="9" t="n"/>
       <c r="K62" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -7156,7 +7156,7 @@
       <c r="J63" s="9" t="n"/>
       <c r="K63" s="9" t="inlineStr">
         <is>
-          <t>ENVS228 PHYSICAL GEOGRAPHY FIELDWORK COURSE (closest)</t>
+          <t>ENVS228 PHYSICAL GEOGRAPHY FIELDWORK COURSE</t>
         </is>
       </c>
     </row>
@@ -7262,7 +7262,7 @@
       <c r="J65" s="10" t="n"/>
       <c r="K65" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -7315,7 +7315,7 @@
       <c r="J66" s="9" t="n"/>
       <c r="K66" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -7474,7 +7474,7 @@
       <c r="J69" s="9" t="n"/>
       <c r="K69" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -7580,7 +7580,7 @@
       <c r="J71" s="9" t="n"/>
       <c r="K71" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -7686,7 +7686,7 @@
       <c r="J73" s="9" t="n"/>
       <c r="K73" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -7792,7 +7792,7 @@
       <c r="J75" s="9" t="n"/>
       <c r="K75" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -7845,7 +7845,7 @@
       <c r="J76" s="9" t="n"/>
       <c r="K76" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -8110,7 +8110,7 @@
       <c r="J81" s="9" t="n"/>
       <c r="K81" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -8163,7 +8163,7 @@
       <c r="J82" s="9" t="n"/>
       <c r="K82" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -8216,7 +8216,7 @@
       <c r="J83" s="9" t="n"/>
       <c r="K83" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -8375,7 +8375,7 @@
       <c r="J86" s="9" t="n"/>
       <c r="K86" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -8428,7 +8428,7 @@
       <c r="J87" s="9" t="n"/>
       <c r="K87" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -8481,7 +8481,7 @@
       <c r="J88" s="9" t="n"/>
       <c r="K88" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -8693,7 +8693,7 @@
       <c r="J92" s="9" t="n"/>
       <c r="K92" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -8746,7 +8746,7 @@
       <c r="J93" s="9" t="n"/>
       <c r="K93" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -8905,7 +8905,7 @@
       <c r="J96" s="10" t="n"/>
       <c r="K96" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -8958,7 +8958,7 @@
       <c r="J97" s="10" t="n"/>
       <c r="K97" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -9117,7 +9117,7 @@
       <c r="J100" s="10" t="n"/>
       <c r="K100" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -9170,7 +9170,7 @@
       <c r="J101" s="10" t="n"/>
       <c r="K101" s="10" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -9276,7 +9276,7 @@
       <c r="J103" s="10" t="n"/>
       <c r="K103" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -9435,7 +9435,7 @@
       <c r="J106" s="10" t="n"/>
       <c r="K106" s="10" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -9594,7 +9594,7 @@
       <c r="J109" s="10" t="n"/>
       <c r="K109" s="10" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -9700,7 +9700,7 @@
       <c r="J111" s="9" t="n"/>
       <c r="K111" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -9753,7 +9753,7 @@
       <c r="J112" s="9" t="n"/>
       <c r="K112" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -9806,7 +9806,7 @@
       <c r="J113" s="9" t="n"/>
       <c r="K113" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -9912,7 +9912,7 @@
       <c r="J115" s="9" t="n"/>
       <c r="K115" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -9965,7 +9965,7 @@
       <c r="J116" s="9" t="n"/>
       <c r="K116" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -10018,7 +10018,7 @@
       <c r="J117" s="9" t="n"/>
       <c r="K117" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -10071,7 +10071,7 @@
       <c r="J118" s="9" t="n"/>
       <c r="K118" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -10124,7 +10124,7 @@
       <c r="J119" s="9" t="n"/>
       <c r="K119" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -10177,7 +10177,7 @@
       <c r="J120" s="9" t="n"/>
       <c r="K120" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -10389,7 +10389,7 @@
       <c r="J124" s="9" t="n"/>
       <c r="K124" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -10442,7 +10442,7 @@
       <c r="J125" s="9" t="n"/>
       <c r="K125" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -10548,7 +10548,7 @@
       <c r="J127" s="9" t="n"/>
       <c r="K127" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -10601,7 +10601,7 @@
       <c r="J128" s="9" t="n"/>
       <c r="K128" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -10707,7 +10707,7 @@
       <c r="J130" s="9" t="n"/>
       <c r="K130" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -10760,7 +10760,7 @@
       <c r="J131" s="9" t="n"/>
       <c r="K131" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -11025,7 +11025,7 @@
       <c r="J136" s="9" t="n"/>
       <c r="K136" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -11131,7 +11131,7 @@
       <c r="J138" s="9" t="n"/>
       <c r="K138" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -11184,7 +11184,7 @@
       <c r="J139" s="9" t="n"/>
       <c r="K139" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -11343,7 +11343,7 @@
       <c r="J142" s="9" t="n"/>
       <c r="K142" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -11396,7 +11396,7 @@
       <c r="J143" s="9" t="n"/>
       <c r="K143" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -11449,7 +11449,7 @@
       <c r="J144" s="9" t="n"/>
       <c r="K144" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -11555,7 +11555,7 @@
       <c r="J146" s="9" t="n"/>
       <c r="K146" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -11661,7 +11661,7 @@
       <c r="J148" s="9" t="n"/>
       <c r="K148" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -11767,7 +11767,7 @@
       <c r="J150" s="9" t="n"/>
       <c r="K150" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -11979,7 +11979,7 @@
       <c r="J154" s="9" t="n"/>
       <c r="K154" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -12032,7 +12032,7 @@
       <c r="J155" s="9" t="n"/>
       <c r="K155" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -12085,7 +12085,7 @@
       <c r="J156" s="9" t="n"/>
       <c r="K156" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -12191,7 +12191,7 @@
       <c r="J158" s="9" t="n"/>
       <c r="K158" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -12403,7 +12403,7 @@
       <c r="J162" s="9" t="n"/>
       <c r="K162" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -12456,7 +12456,7 @@
       <c r="J163" s="9" t="n"/>
       <c r="K163" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -12721,7 +12721,7 @@
       <c r="J168" s="9" t="n"/>
       <c r="K168" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -12774,7 +12774,7 @@
       <c r="J169" s="9" t="n"/>
       <c r="K169" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -13039,7 +13039,7 @@
       <c r="J174" s="9" t="n"/>
       <c r="K174" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -13198,7 +13198,7 @@
       <c r="J177" s="9" t="n"/>
       <c r="K177" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -13251,7 +13251,7 @@
       <c r="J178" s="9" t="n"/>
       <c r="K178" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -13304,7 +13304,7 @@
       <c r="J179" s="9" t="n"/>
       <c r="K179" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -13357,7 +13357,7 @@
       <c r="J180" s="9" t="n"/>
       <c r="K180" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -13410,7 +13410,7 @@
       <c r="J181" s="9" t="n"/>
       <c r="K181" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -13516,7 +13516,7 @@
       <c r="J183" s="9" t="n"/>
       <c r="K183" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -13569,7 +13569,7 @@
       <c r="J184" s="9" t="n"/>
       <c r="K184" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -13728,7 +13728,7 @@
       <c r="J187" s="9" t="n"/>
       <c r="K187" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -13834,7 +13834,7 @@
       <c r="J189" s="9" t="n"/>
       <c r="K189" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -13887,7 +13887,7 @@
       <c r="J190" s="9" t="n"/>
       <c r="K190" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -14099,7 +14099,7 @@
       <c r="J194" s="9" t="n"/>
       <c r="K194" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -14205,7 +14205,7 @@
       <c r="J196" s="9" t="n"/>
       <c r="K196" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -14258,7 +14258,7 @@
       <c r="J197" s="9" t="n"/>
       <c r="K197" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -14311,7 +14311,7 @@
       <c r="J198" s="9" t="n"/>
       <c r="K198" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -14364,7 +14364,7 @@
       <c r="J199" s="9" t="n"/>
       <c r="K199" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -14576,7 +14576,7 @@
       <c r="J203" s="9" t="n"/>
       <c r="K203" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -14682,7 +14682,7 @@
       <c r="J205" s="9" t="n"/>
       <c r="K205" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -14788,7 +14788,7 @@
       <c r="J207" s="9" t="n"/>
       <c r="K207" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -15053,7 +15053,7 @@
       <c r="J212" s="9" t="n"/>
       <c r="K212" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -15106,7 +15106,7 @@
       <c r="J213" s="9" t="n"/>
       <c r="K213" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -15318,7 +15318,7 @@
       <c r="J217" s="9" t="n"/>
       <c r="K217" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -15424,7 +15424,7 @@
       <c r="J219" s="9" t="n"/>
       <c r="K219" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -15530,7 +15530,7 @@
       <c r="J221" s="9" t="n"/>
       <c r="K221" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -15583,7 +15583,7 @@
       <c r="J222" s="9" t="n"/>
       <c r="K222" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -15742,7 +15742,7 @@
       <c r="J225" s="9" t="n"/>
       <c r="K225" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -15795,7 +15795,7 @@
       <c r="J226" s="9" t="n"/>
       <c r="K226" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -15848,7 +15848,7 @@
       <c r="J227" s="9" t="n"/>
       <c r="K227" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -15901,7 +15901,7 @@
       <c r="J228" s="9" t="n"/>
       <c r="K228" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -16007,7 +16007,7 @@
       <c r="J230" s="9" t="n"/>
       <c r="K230" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -16060,7 +16060,7 @@
       <c r="J231" s="9" t="n"/>
       <c r="K231" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -16113,7 +16113,7 @@
       <c r="J232" s="9" t="n"/>
       <c r="K232" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -16537,7 +16537,7 @@
       <c r="J240" s="10" t="n"/>
       <c r="K240" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -16590,7 +16590,7 @@
       <c r="J241" s="10" t="n"/>
       <c r="K241" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -16749,7 +16749,7 @@
       <c r="J244" s="10" t="n"/>
       <c r="K244" s="10" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -16908,7 +16908,7 @@
       <c r="J247" s="10" t="n"/>
       <c r="K247" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -17014,7 +17014,7 @@
       <c r="J249" s="10" t="n"/>
       <c r="K249" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -17385,7 +17385,7 @@
       <c r="J256" s="10" t="n"/>
       <c r="K256" s="10" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -17438,7 +17438,7 @@
       <c r="J257" s="10" t="n"/>
       <c r="K257" s="10" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -17597,7 +17597,7 @@
       <c r="J260" s="9" t="n"/>
       <c r="K260" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -17756,7 +17756,7 @@
       <c r="J263" s="9" t="n"/>
       <c r="K263" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -18074,7 +18074,7 @@
       <c r="J269" s="9" t="n"/>
       <c r="K269" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -18180,7 +18180,7 @@
       <c r="J271" s="9" t="n"/>
       <c r="K271" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -18445,7 +18445,7 @@
       <c r="J276" s="9" t="n"/>
       <c r="K276" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -18498,7 +18498,7 @@
       <c r="J277" s="9" t="n"/>
       <c r="K277" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -18604,7 +18604,7 @@
       <c r="J279" s="9" t="n"/>
       <c r="K279" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -18710,7 +18710,7 @@
       <c r="J281" s="9" t="n"/>
       <c r="K281" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -18763,7 +18763,7 @@
       <c r="J282" s="9" t="n"/>
       <c r="K282" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -18869,7 +18869,7 @@
       <c r="J284" s="9" t="n"/>
       <c r="K284" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -19134,7 +19134,7 @@
       <c r="J289" s="9" t="n"/>
       <c r="K289" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -19187,7 +19187,7 @@
       <c r="J290" s="9" t="n"/>
       <c r="K290" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -19240,7 +19240,7 @@
       <c r="J291" s="9" t="n"/>
       <c r="K291" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -19611,7 +19611,7 @@
       <c r="J298" s="9" t="n"/>
       <c r="K298" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -19664,7 +19664,7 @@
       <c r="J299" s="9" t="n"/>
       <c r="K299" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -19717,7 +19717,7 @@
       <c r="J300" s="9" t="n"/>
       <c r="K300" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -19929,7 +19929,7 @@
       <c r="J304" s="9" t="n"/>
       <c r="K304" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -20088,7 +20088,7 @@
       <c r="J307" s="9" t="n"/>
       <c r="K307" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -20141,7 +20141,7 @@
       <c r="J308" s="9" t="n"/>
       <c r="K308" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -20194,7 +20194,7 @@
       <c r="J309" s="9" t="n"/>
       <c r="K309" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -20353,7 +20353,7 @@
       <c r="J312" s="9" t="n"/>
       <c r="K312" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -20406,7 +20406,7 @@
       <c r="J313" s="9" t="n"/>
       <c r="K313" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -20512,7 +20512,7 @@
       <c r="J315" s="9" t="n"/>
       <c r="K315" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -20671,7 +20671,7 @@
       <c r="J318" s="9" t="n"/>
       <c r="K318" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -20724,7 +20724,7 @@
       <c r="J319" s="9" t="n"/>
       <c r="K319" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -20883,7 +20883,7 @@
       <c r="J322" s="9" t="n"/>
       <c r="K322" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -21095,7 +21095,7 @@
       <c r="J326" s="9" t="n"/>
       <c r="K326" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -21148,7 +21148,7 @@
       <c r="J327" s="9" t="n"/>
       <c r="K327" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -21307,7 +21307,7 @@
       <c r="J330" s="9" t="n"/>
       <c r="K330" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -21360,7 +21360,7 @@
       <c r="J331" s="9" t="n"/>
       <c r="K331" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -21466,7 +21466,7 @@
       <c r="J333" s="9" t="n"/>
       <c r="K333" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -21519,7 +21519,7 @@
       <c r="J334" s="9" t="n"/>
       <c r="K334" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -21572,7 +21572,7 @@
       <c r="J335" s="9" t="n"/>
       <c r="K335" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -21678,7 +21678,7 @@
       <c r="J337" s="12" t="n"/>
       <c r="K337" s="12" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -21943,7 +21943,7 @@
       <c r="J342" s="12" t="n"/>
       <c r="K342" s="12" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -22102,7 +22102,7 @@
       <c r="J345" s="9" t="n"/>
       <c r="K345" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -22155,7 +22155,7 @@
       <c r="J346" s="9" t="n"/>
       <c r="K346" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -22208,7 +22208,7 @@
       <c r="J347" s="9" t="n"/>
       <c r="K347" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -22632,7 +22632,7 @@
       <c r="J355" s="9" t="n"/>
       <c r="K355" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -22791,7 +22791,7 @@
       <c r="J358" s="9" t="n"/>
       <c r="K358" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -22844,7 +22844,7 @@
       <c r="J359" s="9" t="n"/>
       <c r="K359" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -22950,7 +22950,7 @@
       <c r="J361" s="9" t="n"/>
       <c r="K361" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -23056,7 +23056,7 @@
       <c r="J363" s="9" t="n"/>
       <c r="K363" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -23109,7 +23109,7 @@
       <c r="J364" s="9" t="n"/>
       <c r="K364" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -23215,7 +23215,7 @@
       <c r="J366" s="9" t="n"/>
       <c r="K366" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -23427,7 +23427,7 @@
       <c r="J370" s="9" t="n"/>
       <c r="K370" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -23586,7 +23586,7 @@
       <c r="J373" s="9" t="n"/>
       <c r="K373" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -23692,7 +23692,7 @@
       <c r="J375" s="9" t="n"/>
       <c r="K375" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -23851,7 +23851,7 @@
       <c r="J378" s="9" t="n"/>
       <c r="K378" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -23957,7 +23957,7 @@
       <c r="J380" s="9" t="n"/>
       <c r="K380" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -24010,7 +24010,7 @@
       <c r="J381" s="9" t="n"/>
       <c r="K381" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -24116,7 +24116,7 @@
       <c r="J383" s="9" t="n"/>
       <c r="K383" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -24169,7 +24169,7 @@
       <c r="J384" s="9" t="n"/>
       <c r="K384" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -24275,7 +24275,7 @@
       <c r="J386" s="9" t="n"/>
       <c r="K386" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -24805,7 +24805,7 @@
       <c r="J396" s="9" t="n"/>
       <c r="K396" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -24911,7 +24911,7 @@
       <c r="J398" s="9" t="n"/>
       <c r="K398" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -25123,7 +25123,7 @@
       <c r="J402" s="12" t="n"/>
       <c r="K402" s="12" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -25176,7 +25176,7 @@
       <c r="J403" s="9" t="n"/>
       <c r="K403" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -25441,7 +25441,7 @@
       <c r="J408" s="9" t="n"/>
       <c r="K408" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -25494,7 +25494,7 @@
       <c r="J409" s="9" t="n"/>
       <c r="K409" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -25918,7 +25918,7 @@
       <c r="J417" s="9" t="n"/>
       <c r="K417" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -25971,7 +25971,7 @@
       <c r="J418" s="9" t="n"/>
       <c r="K418" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -26024,7 +26024,7 @@
       <c r="J419" s="9" t="n"/>
       <c r="K419" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -26183,7 +26183,7 @@
       <c r="J422" s="10" t="n"/>
       <c r="K422" s="10" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -26236,7 +26236,7 @@
       <c r="J423" s="10" t="n"/>
       <c r="K423" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -26289,7 +26289,7 @@
       <c r="J424" s="10" t="n"/>
       <c r="K424" s="10" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -26342,7 +26342,7 @@
       <c r="J425" s="10" t="n"/>
       <c r="K425" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -26395,7 +26395,7 @@
       <c r="J426" s="10" t="n"/>
       <c r="K426" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -26501,7 +26501,7 @@
       <c r="J428" s="10" t="n"/>
       <c r="K428" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -26713,7 +26713,7 @@
       <c r="J432" s="10" t="n"/>
       <c r="K432" s="10" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -26872,7 +26872,7 @@
       <c r="J435" s="10" t="n"/>
       <c r="K435" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -26925,7 +26925,7 @@
       <c r="J436" s="10" t="n"/>
       <c r="K436" s="10" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -27137,7 +27137,7 @@
       <c r="J440" s="10" t="n"/>
       <c r="K440" s="10" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -27190,7 +27190,7 @@
       <c r="J441" s="10" t="n"/>
       <c r="K441" s="10" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -27243,7 +27243,7 @@
       <c r="J442" s="10" t="n"/>
       <c r="K442" s="10" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -27296,7 +27296,7 @@
       <c r="J443" s="10" t="n"/>
       <c r="K443" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -27667,7 +27667,7 @@
       <c r="J450" s="9" t="n"/>
       <c r="K450" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -27826,7 +27826,7 @@
       <c r="J453" s="9" t="n"/>
       <c r="K453" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -27985,7 +27985,7 @@
       <c r="J456" s="9" t="n"/>
       <c r="K456" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -28091,7 +28091,7 @@
       <c r="J458" s="9" t="n"/>
       <c r="K458" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -28144,7 +28144,7 @@
       <c r="J459" s="9" t="n"/>
       <c r="K459" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -28197,7 +28197,7 @@
       <c r="J460" s="9" t="n"/>
       <c r="K460" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -28250,7 +28250,7 @@
       <c r="J461" s="9" t="n"/>
       <c r="K461" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -28356,7 +28356,7 @@
       <c r="J463" s="9" t="n"/>
       <c r="K463" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -28409,7 +28409,7 @@
       <c r="J464" s="12" t="n"/>
       <c r="K464" s="12" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -28674,7 +28674,7 @@
       <c r="J469" s="12" t="n"/>
       <c r="K469" s="12" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -28886,7 +28886,7 @@
       <c r="J473" s="9" t="n"/>
       <c r="K473" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -28992,7 +28992,7 @@
       <c r="J475" s="9" t="n"/>
       <c r="K475" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -29045,7 +29045,7 @@
       <c r="J476" s="9" t="n"/>
       <c r="K476" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -29098,7 +29098,7 @@
       <c r="J477" s="9" t="n"/>
       <c r="K477" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -29151,7 +29151,7 @@
       <c r="J478" s="9" t="n"/>
       <c r="K478" s="9" t="inlineStr">
         <is>
-          <t>ENVS228 PHYSICAL GEOGRAPHY FIELDWORK COURSE (closest)</t>
+          <t>ENVS228 PHYSICAL GEOGRAPHY FIELDWORK COURSE</t>
         </is>
       </c>
     </row>
@@ -29416,7 +29416,7 @@
       <c r="J483" s="9" t="n"/>
       <c r="K483" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -29469,7 +29469,7 @@
       <c r="J484" s="9" t="n"/>
       <c r="K484" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -29522,7 +29522,7 @@
       <c r="J485" s="9" t="n"/>
       <c r="K485" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -29575,7 +29575,7 @@
       <c r="J486" s="9" t="n"/>
       <c r="K486" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -29840,7 +29840,7 @@
       <c r="J491" s="9" t="n"/>
       <c r="K491" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -29893,7 +29893,7 @@
       <c r="J492" s="9" t="n"/>
       <c r="K492" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -29946,7 +29946,7 @@
       <c r="J493" s="9" t="n"/>
       <c r="K493" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -29999,7 +29999,7 @@
       <c r="J494" s="9" t="n"/>
       <c r="K494" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -30158,7 +30158,7 @@
       <c r="J497" s="9" t="n"/>
       <c r="K497" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -30211,7 +30211,7 @@
       <c r="J498" s="9" t="n"/>
       <c r="K498" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -30317,7 +30317,7 @@
       <c r="J500" s="9" t="n"/>
       <c r="K500" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -30370,7 +30370,7 @@
       <c r="J501" s="9" t="n"/>
       <c r="K501" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -30529,7 +30529,7 @@
       <c r="J504" s="9" t="n"/>
       <c r="K504" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -30582,7 +30582,7 @@
       <c r="J505" s="9" t="n"/>
       <c r="K505" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -30688,7 +30688,7 @@
       <c r="J507" s="9" t="n"/>
       <c r="K507" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -30847,7 +30847,7 @@
       <c r="J510" s="9" t="n"/>
       <c r="K510" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -30900,7 +30900,7 @@
       <c r="J511" s="9" t="n"/>
       <c r="K511" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -31165,7 +31165,7 @@
       <c r="J516" s="9" t="n"/>
       <c r="K516" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -31218,7 +31218,7 @@
       <c r="J517" s="9" t="n"/>
       <c r="K517" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -31271,7 +31271,7 @@
       <c r="J518" s="9" t="n"/>
       <c r="K518" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -31324,7 +31324,7 @@
       <c r="J519" s="9" t="n"/>
       <c r="K519" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -31589,7 +31589,7 @@
       <c r="J524" s="9" t="n"/>
       <c r="K524" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -31642,7 +31642,7 @@
       <c r="J525" s="9" t="n"/>
       <c r="K525" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -31748,7 +31748,7 @@
       <c r="J527" s="9" t="n"/>
       <c r="K527" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -32119,7 +32119,7 @@
       <c r="J534" s="9" t="n"/>
       <c r="K534" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -32172,7 +32172,7 @@
       <c r="J535" s="9" t="n"/>
       <c r="K535" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -32225,7 +32225,7 @@
       <c r="J536" s="9" t="n"/>
       <c r="K536" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -32331,7 +32331,7 @@
       <c r="J538" s="9" t="n"/>
       <c r="K538" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -32384,7 +32384,7 @@
       <c r="J539" s="9" t="n"/>
       <c r="K539" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -32702,7 +32702,7 @@
       <c r="J545" s="9" t="n"/>
       <c r="K545" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -32808,7 +32808,7 @@
       <c r="J547" s="9" t="n"/>
       <c r="K547" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -32861,7 +32861,7 @@
       <c r="J548" s="9" t="n"/>
       <c r="K548" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -33126,7 +33126,7 @@
       <c r="J553" s="9" t="n"/>
       <c r="K553" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -33232,7 +33232,7 @@
       <c r="J555" s="10" t="n"/>
       <c r="K555" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -33285,7 +33285,7 @@
       <c r="J556" s="10" t="n"/>
       <c r="K556" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -33338,7 +33338,7 @@
       <c r="J557" s="10" t="n"/>
       <c r="K557" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -33391,7 +33391,7 @@
       <c r="J558" s="10" t="n"/>
       <c r="K558" s="10" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -33497,7 +33497,7 @@
       <c r="J560" s="10" t="n"/>
       <c r="K560" s="10" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -33603,7 +33603,7 @@
       <c r="J562" s="10" t="n"/>
       <c r="K562" s="10" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -33656,7 +33656,7 @@
       <c r="J563" s="10" t="n"/>
       <c r="K563" s="10" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -33762,7 +33762,7 @@
       <c r="J565" s="10" t="n"/>
       <c r="K565" s="10" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -34027,7 +34027,7 @@
       <c r="J570" s="10" t="n"/>
       <c r="K570" s="10" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -34080,7 +34080,7 @@
       <c r="J571" s="10" t="n"/>
       <c r="K571" s="10" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -34292,7 +34292,7 @@
       <c r="J575" s="10" t="n"/>
       <c r="K575" s="10" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -34345,7 +34345,7 @@
       <c r="J576" s="9" t="n"/>
       <c r="K576" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -34398,7 +34398,7 @@
       <c r="J577" s="9" t="n"/>
       <c r="K577" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -34663,7 +34663,7 @@
       <c r="J582" s="9" t="n"/>
       <c r="K582" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -34716,7 +34716,7 @@
       <c r="J583" s="9" t="n"/>
       <c r="K583" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -34981,7 +34981,7 @@
       <c r="J588" s="9" t="n"/>
       <c r="K588" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -35034,7 +35034,7 @@
       <c r="J589" s="9" t="n"/>
       <c r="K589" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -35087,7 +35087,7 @@
       <c r="J590" s="9" t="n"/>
       <c r="K590" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -35193,7 +35193,7 @@
       <c r="J592" s="9" t="n"/>
       <c r="K592" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -35246,7 +35246,7 @@
       <c r="J593" s="9" t="n"/>
       <c r="K593" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -35299,7 +35299,7 @@
       <c r="J594" s="9" t="n"/>
       <c r="K594" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -35458,7 +35458,7 @@
       <c r="J597" s="9" t="n"/>
       <c r="K597" s="9" t="inlineStr">
         <is>
-          <t>ENVS228 PHYSICAL GEOGRAPHY FIELDWORK COURSE (closest)</t>
+          <t>ENVS228 PHYSICAL GEOGRAPHY FIELDWORK COURSE</t>
         </is>
       </c>
     </row>
@@ -35617,7 +35617,7 @@
       <c r="J600" s="9" t="n"/>
       <c r="K600" s="9" t="inlineStr">
         <is>
-          <t>ENVS228 PHYSICAL GEOGRAPHY FIELDWORK COURSE (closest)</t>
+          <t>ENVS228 PHYSICAL GEOGRAPHY FIELDWORK COURSE</t>
         </is>
       </c>
     </row>
@@ -35988,7 +35988,7 @@
       <c r="J607" s="9" t="n"/>
       <c r="K607" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -36041,7 +36041,7 @@
       <c r="J608" s="9" t="n"/>
       <c r="K608" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -36200,7 +36200,7 @@
       <c r="J611" s="9" t="n"/>
       <c r="K611" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -36465,7 +36465,7 @@
       <c r="J616" s="9" t="n"/>
       <c r="K616" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -36518,7 +36518,7 @@
       <c r="J617" s="9" t="n"/>
       <c r="K617" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -36571,7 +36571,7 @@
       <c r="J618" s="9" t="n"/>
       <c r="K618" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -36624,7 +36624,7 @@
       <c r="J619" s="9" t="n"/>
       <c r="K619" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -36677,7 +36677,7 @@
       <c r="J620" s="9" t="n"/>
       <c r="K620" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -36783,7 +36783,7 @@
       <c r="J622" s="9" t="n"/>
       <c r="K622" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -36995,7 +36995,7 @@
       <c r="J626" s="9" t="n"/>
       <c r="K626" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -37101,7 +37101,7 @@
       <c r="J628" s="9" t="n"/>
       <c r="K628" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -37154,7 +37154,7 @@
       <c r="J629" s="9" t="n"/>
       <c r="K629" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -37207,7 +37207,7 @@
       <c r="J630" s="9" t="n"/>
       <c r="K630" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -37260,7 +37260,7 @@
       <c r="J631" s="9" t="n"/>
       <c r="K631" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -37366,7 +37366,7 @@
       <c r="J633" s="9" t="n"/>
       <c r="K633" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -37419,7 +37419,7 @@
       <c r="J634" s="9" t="n"/>
       <c r="K634" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -37472,7 +37472,7 @@
       <c r="J635" s="9" t="n"/>
       <c r="K635" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -37578,7 +37578,7 @@
       <c r="J637" s="9" t="n"/>
       <c r="K637" s="9" t="inlineStr">
         <is>
-          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION (closest)</t>
+          <t>ENVS264 POLITICAL ECONOMIES OF GLOBALISATION</t>
         </is>
       </c>
     </row>
@@ -37631,7 +37631,7 @@
       <c r="J638" s="9" t="n"/>
       <c r="K638" s="9" t="inlineStr">
         <is>
-          <t>ENVS223 AN INTRODUCTION TO ENVIRONMENTAL HISTORY (closest - new module, no direct equivalent)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -37843,7 +37843,7 @@
       <c r="J642" s="9" t="n"/>
       <c r="K642" s="9" t="inlineStr">
         <is>
-          <t>ENVS231 CLIMATOLOGY / ENVS217 CATCHMENT HYDROLOGY (closest)</t>
+          <t>ENVS217 CATCHMENT HYDROLOGY</t>
         </is>
       </c>
     </row>
@@ -38002,7 +38002,7 @@
       <c r="J645" s="9" t="n"/>
       <c r="K645" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -38055,7 +38055,7 @@
       <c r="J646" s="9" t="n"/>
       <c r="K646" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -38108,7 +38108,7 @@
       <c r="J647" s="9" t="n"/>
       <c r="K647" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -38161,7 +38161,7 @@
       <c r="J648" s="9" t="n"/>
       <c r="K648" s="9" t="inlineStr">
         <is>
-          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY (closest)</t>
+          <t>ENVS218 PLANNING FOR ENVIRONMENTAL SUSTAINABILITY</t>
         </is>
       </c>
     </row>
@@ -38214,7 +38214,7 @@
       <c r="J649" s="9" t="n"/>
       <c r="K649" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -38267,7 +38267,7 @@
       <c r="J650" s="9" t="n"/>
       <c r="K650" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -38320,7 +38320,7 @@
       <c r="J651" s="9" t="n"/>
       <c r="K651" s="9" t="inlineStr">
         <is>
-          <t>ENVS257 GIS FOR HUMAN GEOGRAPHY (closest - no physical-geography GIS module in Year 2)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -38373,7 +38373,7 @@
       <c r="J652" s="9" t="n"/>
       <c r="K652" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>
@@ -38479,7 +38479,7 @@
       <c r="J654" s="9" t="n"/>
       <c r="K654" s="9" t="inlineStr">
         <is>
-          <t>ENVS205 PEOPLE AND PLACE (closest)</t>
+          <t>No ENVS equivalent (new module)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix semester text on UTD GISC4381 core row; 4000-level US courses as Level 4
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EZa6h9SpqLeB7ZbHz6KiwN
</commit_message>
<xml_diff>
--- a/curriculum_mapping_2026-27/20261013_CurriculumMapping_Geography.xlsx
+++ b/curriculum_mapping_2026-27/20261013_CurriculumMapping_Geography.xlsx
@@ -5350,7 +5350,7 @@
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>Not confirmed</t>
+          <t>Fall 2026</t>
         </is>
       </c>
       <c r="I29" s="12" t="inlineStr">
@@ -19703,7 +19703,7 @@
       </c>
       <c r="F300" s="9" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 4</t>
         </is>
       </c>
       <c r="G300" s="9" t="inlineStr">
@@ -21876,7 +21876,7 @@
       </c>
       <c r="F341" s="9" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 4</t>
         </is>
       </c>
       <c r="G341" s="9" t="inlineStr">
@@ -21929,7 +21929,7 @@
       </c>
       <c r="F342" s="9" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 4</t>
         </is>
       </c>
       <c r="G342" s="9" t="inlineStr">
@@ -31787,7 +31787,7 @@
       </c>
       <c r="F528" s="9" t="inlineStr">
         <is>
-          <t>Level 3</t>
+          <t>Level 4</t>
         </is>
       </c>
       <c r="G528" s="9" t="inlineStr">

</xml_diff>